<commit_message>
Complete Z isomer G1 SPE shieldings; full DP4+ H+13C and Excel tables
Co-authored-by: mehmetalagoz <mehmetalagoz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dp4_oxime/DP4_Sarotti_ZoneB_giris.xlsx
+++ b/dp4_oxime/DP4_Sarotti_ZoneB_giris.xlsx
@@ -14,30 +14,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="43">
   <si>
     <t>Nuclei</t>
   </si>
   <si>
-    <t>sp2_x</t>
-  </si>
-  <si>
-    <t>Exp_ppm</t>
+    <t>sp2 (x if sp2)</t>
+  </si>
+  <si>
+    <t>Experimental (ppm)</t>
   </si>
   <si>
     <t>Assignment</t>
   </si>
   <si>
-    <t>E_atoms</t>
-  </si>
-  <si>
-    <t>sigma_E</t>
-  </si>
-  <si>
-    <t>Z_atoms</t>
-  </si>
-  <si>
-    <t>sigma_Z</t>
+    <t>E atom(s)</t>
+  </si>
+  <si>
+    <t>sigma E (shielding)</t>
+  </si>
+  <si>
+    <t>Z atom(s)</t>
+  </si>
+  <si>
+    <t>sigma Z (shielding)</t>
   </si>
   <si>
     <t>H</t>
@@ -64,7 +64,7 @@
     <t>Phenyl</t>
   </si>
   <si>
-    <t>C=N oxime</t>
+    <t>C=N (oxime)</t>
   </si>
   <si>
     <t>Aromatic quat.</t>
@@ -73,22 +73,19 @@
     <t>Aromatic</t>
   </si>
   <si>
-    <t>Aromatic / pyrazole</t>
-  </si>
-  <si>
     <t>Aromatic CH</t>
   </si>
   <si>
     <t>Pyrazole CH</t>
   </si>
   <si>
-    <t>H24,H25,H26</t>
-  </si>
-  <si>
-    <t>H30,H31,H32</t>
-  </si>
-  <si>
-    <t>H21,H22</t>
+    <t>H24, H25, H26</t>
+  </si>
+  <si>
+    <t>H30, H31, H32</t>
+  </si>
+  <si>
+    <t>H21, H22</t>
   </si>
   <si>
     <t>H23</t>
@@ -97,10 +94,10 @@
     <t>H27</t>
   </si>
   <si>
-    <t>H19,H20</t>
-  </si>
-  <si>
-    <t>H28,H29</t>
+    <t>H19, H20</t>
+  </si>
+  <si>
+    <t>H28, H29</t>
   </si>
   <si>
     <t>C6</t>
@@ -133,7 +130,16 @@
     <t>C11</t>
   </si>
   <si>
-    <t>H28,H29,H30</t>
+    <t>H28, H29, H30</t>
+  </si>
+  <si>
+    <t>H31, H32</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>C3</t>
   </si>
   <si>
     <t>C16</t>
@@ -508,13 +514,13 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2">
-        <v>29.927967</v>
+        <v>29.92376666666667</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2">
         <v>29.77</v>
@@ -531,16 +537,16 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F3">
-        <v>27.752433</v>
+        <v>27.75243333333333</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H3">
-        <v>27.55</v>
+        <v>27.55186666666667</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -554,16 +560,16 @@
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F4">
         <v>26.65465</v>
       </c>
       <c r="G4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H4">
-        <v>26.65</v>
+        <v>26.6476</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -580,16 +586,16 @@
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F5">
         <v>24.5065</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H5">
-        <v>23.941</v>
+        <v>23.9358</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -606,16 +612,16 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F6">
         <v>24.6019</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H6">
-        <v>24.4462</v>
+        <v>24.4461</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -632,16 +638,16 @@
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F7">
         <v>24.26725</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H7">
-        <v>23.8193</v>
+        <v>23.81635</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -658,16 +664,16 @@
         <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F8">
         <v>23.9462</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H8">
-        <v>24.0887</v>
+        <v>24.0934</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -684,13 +690,16 @@
         <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F9">
         <v>42.2965</v>
       </c>
       <c r="G9" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="H9">
+        <v>40.5692</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -707,13 +716,16 @@
         <v>17</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F10">
         <v>52.1827</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="H10">
+        <v>52.0531</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -730,13 +742,16 @@
         <v>18</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11">
         <v>58.1784</v>
       </c>
       <c r="G11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="H11">
+        <v>58.0842</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -753,13 +768,16 @@
         <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F12">
         <v>62.9938</v>
       </c>
       <c r="G12" t="s">
         <v>32</v>
+      </c>
+      <c r="H12">
+        <v>66.5826</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -773,16 +791,19 @@
         <v>127.43</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F13">
         <v>65.7726</v>
       </c>
       <c r="G13" t="s">
-        <v>33</v>
+        <v>40</v>
+      </c>
+      <c r="H13">
+        <v>67.2871</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -796,16 +817,19 @@
         <v>126.84</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F14">
         <v>66.8511</v>
       </c>
       <c r="G14" t="s">
-        <v>34</v>
+        <v>41</v>
+      </c>
+      <c r="H14">
+        <v>67.7131</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -819,16 +843,19 @@
         <v>115.74</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F15">
         <v>74.7594</v>
       </c>
       <c r="G15" t="s">
-        <v>35</v>
+        <v>34</v>
+      </c>
+      <c r="H15">
+        <v>75.0134</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -842,16 +869,19 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F16">
         <v>130.8007</v>
       </c>
       <c r="G16" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>42</v>
+      </c>
+      <c r="H16">
+        <v>130.3561</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -862,16 +892,19 @@
         <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F17">
         <v>135.9479</v>
       </c>
       <c r="G17" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+        <v>36</v>
+      </c>
+      <c r="H17">
+        <v>145.1832</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -882,13 +915,16 @@
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F18">
         <v>181.286</v>
       </c>
       <c r="G18" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="H18">
+        <v>181.2012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>